<commit_message>
feat: feedback R1 — niveles, talleres extra, vista del director, portal del ejecutivo y contacto
- Niveles escolares por colegio (chips) y nivel por servicio (select + badge)
- Talleres extra de coordinación (+Uso/+Prof/+Didáctica, badge EXTRA, quitables)
- Vista del director: enlace público #/director/<token> (revocable) con página
  de avance sanitizada (RPC psp_vista_director) + vista previa interna
- 5º rol 'ejecutivo': portal /mis-colegios solo lectura con énfasis en
  comentarios y reportes del asesor
- Contacto del colegio (nombre/rol/tel/correo) en tarjeta, portales y carga BI
- Plantilla BI: columnas Niveles y Contacto; parser con derivación de niveles
- SQL: supabase_actualizacion_v3_1.sql (rol, trigger, RPC público)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-colegios.xlsx
+++ b/public/plantilla-colegios.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:X4"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -410,15 +410,20 @@
     <col min="8" max="8" width="23.83203125" customWidth="1"/>
     <col min="9" max="9" width="19.83203125" customWidth="1"/>
     <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="19.83203125" customWidth="1"/>
-    <col min="16" max="16" width="17.83203125" customWidth="1"/>
-    <col min="17" max="17" width="19.83203125" customWidth="1"/>
-    <col min="18" max="18" width="21.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="19.83203125" customWidth="1"/>
+    <col min="17" max="17" width="17.83203125" customWidth="1"/>
+    <col min="18" max="18" width="19.83203125" customWidth="1"/>
+    <col min="19" max="19" width="21.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="19.83203125" customWidth="1"/>
+    <col min="24" max="24" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,31 +458,46 @@
         <v>Años de Antigüedad</v>
       </c>
       <c r="K1" t="str">
+        <v>Niveles</v>
+      </c>
+      <c r="L1" t="str">
         <v>Serie Preescolar</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Serie Primaria</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Serie Secundaria</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Bachillerato</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Inglés Preescolar</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Inglés Primaria</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Inglés Secundaria</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Inglés Bachillerato</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Otra Serie</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Contacto Nombre</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Contacto Rol</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Contacto Teléfono</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Contacto Correo</v>
       </c>
     </row>
     <row r="2">
@@ -512,7 +532,7 @@
         <v>12</v>
       </c>
       <c r="K2" t="str">
-        <v>Acierta</v>
+        <v>Preescolar, Primaria, Secundaria</v>
       </c>
       <c r="L2" t="str">
         <v>Acierta</v>
@@ -521,22 +541,37 @@
         <v>Acierta</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>Acierta</v>
       </c>
       <c r="O2" t="str">
-        <v>Bright Sparks</v>
+        <v/>
       </c>
       <c r="P2" t="str">
         <v>Bright Sparks</v>
       </c>
       <c r="Q2" t="str">
+        <v>Bright Sparks</v>
+      </c>
+      <c r="R2" t="str">
         <v>Winglish</v>
       </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
       <c r="S2" t="str">
         <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v>Gabriela Rentería</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Directora académica</v>
+      </c>
+      <c r="W2" t="str">
+        <v>55 1234 5678</v>
+      </c>
+      <c r="X2" t="str">
+        <v>g.renteria@cumbresvalle.edu.mx</v>
       </c>
     </row>
     <row r="3">
@@ -571,31 +606,46 @@
         <v>5</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>Primaria, Secundaria</v>
       </c>
       <c r="L3" t="str">
-        <v>Revuela Up</v>
+        <v/>
       </c>
       <c r="M3" t="str">
         <v>Revuela Up</v>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>Revuela Up</v>
       </c>
       <c r="O3" t="str">
         <v/>
       </c>
       <c r="P3" t="str">
-        <v>Winglish</v>
+        <v/>
       </c>
       <c r="Q3" t="str">
         <v>Winglish</v>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>Winglish</v>
       </c>
       <c r="S3" t="str">
         <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v>Raúl Ortega</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Coordinador general</v>
+      </c>
+      <c r="W3" t="str">
+        <v>81 9876 5432</v>
+      </c>
+      <c r="X3" t="str">
+        <v>rortega@nuevoamanecer.mx</v>
       </c>
     </row>
     <row r="4">
@@ -633,11 +683,11 @@
         <v/>
       </c>
       <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>Revuela Up</v>
       </c>
-      <c r="M4" t="str">
-        <v/>
-      </c>
       <c r="N4" t="str">
         <v/>
       </c>
@@ -654,19 +704,34 @@
         <v/>
       </c>
       <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
         <v>Serie legada 2019</v>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D28"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -811,7 +876,7 @@
         <v>Texto (nombre completo)</v>
       </c>
       <c r="D10" t="str">
-        <v>Asesor que atiende los servicios académicos. Se convierte en el asesor del colegio: si no existe se crea y el colegio queda asignado a él.</v>
+        <v>Asesor que atiende los servicios pedagógicos. Se convierte en el asesor del colegio: si no existe se crea y el colegio queda asignado a él.</v>
       </c>
     </row>
     <row r="11">
@@ -830,21 +895,21 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Serie Preescolar</v>
+        <v>Niveles</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
       </c>
       <c r="C12" t="str">
-        <v>Texto</v>
+        <v>Lista separada por comas</v>
       </c>
       <c r="D12" t="str">
-        <v>Serie que usa en ese nivel (vacío = no aplica).</v>
+        <v>Niveles escolares del colegio: Preescolar, Primaria, Secundaria y/o Bachillerato. Si viene vacía, se deducen de las columnas de serie/inglés por nivel.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Serie Primaria</v>
+        <v>Serie Preescolar</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
@@ -853,12 +918,12 @@
         <v>Texto</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>Serie que usa en ese nivel (vacío = no aplica).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Serie Secundaria</v>
+        <v>Serie Primaria</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
@@ -872,7 +937,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Bachillerato</v>
+        <v>Serie Secundaria</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
@@ -881,12 +946,12 @@
         <v>Texto</v>
       </c>
       <c r="D15" t="str">
-        <v>Serie de bachillerato (vacío = no aplica).</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Inglés Preescolar</v>
+        <v>Bachillerato</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
@@ -895,12 +960,12 @@
         <v>Texto</v>
       </c>
       <c r="D16" t="str">
-        <v>Programa de inglés en ese nivel.</v>
+        <v>Serie de bachillerato (vacío = no aplica).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Inglés Primaria</v>
+        <v>Inglés Preescolar</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
@@ -909,12 +974,12 @@
         <v>Texto</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>Programa de inglés en ese nivel.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Inglés Secundaria</v>
+        <v>Inglés Primaria</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
@@ -928,7 +993,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Inglés Bachillerato</v>
+        <v>Inglés Secundaria</v>
       </c>
       <c r="B19" t="str">
         <v>No</v>
@@ -942,7 +1007,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Otra Serie</v>
+        <v>Inglés Bachillerato</v>
       </c>
       <c r="B20" t="str">
         <v>No</v>
@@ -951,40 +1016,110 @@
         <v>Texto</v>
       </c>
       <c r="D20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Otra Serie</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D21" t="str">
         <v>Cualquier otra serie no contemplada arriba.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Formato</v>
+        <v>Contacto Nombre</v>
       </c>
       <c r="B22" t="str">
-        <v/>
+        <v>Recomendada</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>Texto</v>
       </c>
       <c r="D22" t="str">
-        <v>Una fila por colegio. No cambiar los encabezados. Se acepta .xlsx o .csv (UTF-8).</v>
+        <v>Persona del colegio con quien se coordinan la agenda y la prestación de servicios.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Contacto Rol</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Recomendada</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Cargo del contacto (directora académica, coordinador general…).</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Contacto Teléfono</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Recomendada</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Teléfono directo del contacto.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Contacto Correo</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Recomendada</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Correo</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Correo del contacto.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Formato</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v>Una fila por colegio. No cambiar los encabezados. Se acepta .xlsx o .csv (UTF-8).</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Ejemplos</v>
       </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v/>
-      </c>
-      <c r="D23" t="str">
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
         <v>Las 3 filas de la hoja «Colegios» son de ejemplo: bórrenlas antes de entregar.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>